<commit_message>
Restaurado criterio tnut 2024: primer time_h > 0. Redondeo de temperatura de diseño a entero y tnut a múltiplos de 6 h. condition_id actualizado (RICH_T{T}_A{tnut}h / CCD_T{T}_tnut{tnut}h). Cálculo tnut 2025 usando chem_df25 (Código → timestamp adición). Cálculo tnut 2024 desde chem_df interno (ignora time_h ≤ 0). Añadidos diagnósticos detallados (T_mean, tnut raw vs redondeado). Mantención de replicate_id por (year, condition_id). Integración fallback de temperatura 2025 desde archivos externos. Ajuste sobre datos experimentales para cuadrar bien tiempos de nutrición y adición de nutrientes de por si.
</commit_message>
<xml_diff>
--- a/Datos Experimentales/Data 24024.xlsx
+++ b/Datos Experimentales/Data 24024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cltor\Documents\SB_Calibration_2025\Datos Experimentales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72544A3-4BA4-4A67-B90C-AD9B52B35AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1A9B9D-6D90-499B-B0D6-152505E876E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Antecedentes_info" sheetId="1" r:id="rId1"/>
@@ -1431,9 +1431,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B117"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -1569,7 +1569,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1585,7 +1585,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -1609,7 +1609,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>31</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1681,7 +1681,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1737,7 +1737,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1761,7 +1761,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -1825,7 +1825,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -1841,7 +1841,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>62</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>63</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>64</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>65</v>
       </c>
@@ -1897,7 +1897,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>67</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>68</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -1921,7 +1921,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -1929,7 +1929,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>71</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>72</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>74</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>75</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>77</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>78</v>
       </c>
@@ -1985,7 +1985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>80</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>81</v>
       </c>
@@ -2009,7 +2009,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>82</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>84</v>
       </c>
@@ -2033,7 +2033,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>85</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>87</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>88</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>90</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>91</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>92</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>94</v>
       </c>
@@ -2097,7 +2097,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>95</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>96</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>97</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>98</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>99</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>100</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>101</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>102</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>103</v>
       </c>
@@ -2169,7 +2169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>104</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>105</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>106</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>107</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>108</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>110</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>111</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>113</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>114</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>115</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>116</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>117</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>118</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>119</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>120</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>121</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>122</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>123</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>124</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>126</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>127</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>128</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>129</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>130</v>
       </c>
@@ -2380,7 +2380,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -2392,9 +2392,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>281</v>
       </c>
@@ -2425,9 +2425,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>286</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>289</v>
       </c>
@@ -2449,7 +2449,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>290</v>
       </c>
@@ -2460,7 +2460,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>291</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>292</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>293</v>
       </c>
@@ -2493,7 +2493,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>294</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>295</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>297</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>298</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>299</v>
       </c>
@@ -2559,7 +2559,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>300</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>301</v>
       </c>
@@ -2581,7 +2581,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>302</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>303</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>304</v>
       </c>
@@ -2614,7 +2614,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>305</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>306</v>
       </c>
@@ -2636,7 +2636,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>307</v>
       </c>
@@ -2647,7 +2647,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>308</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>309</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>15.9</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>310</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>15.8</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>311</v>
       </c>
@@ -2691,7 +2691,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>312</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>313</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>314</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>16.399999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>315</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>316</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>317</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>318</v>
       </c>
@@ -2768,7 +2768,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>319</v>
       </c>
@@ -2779,7 +2779,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>320</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>321</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>322</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>323</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>324</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>325</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>326</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>327</v>
       </c>
@@ -2867,7 +2867,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>328</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>329</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>330</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>331</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>332</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>333</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>334</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>335</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>16.100000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>336</v>
       </c>
@@ -2977,9 +2977,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>286</v>
       </c>
@@ -2990,7 +2993,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>289</v>
       </c>
@@ -3001,7 +3004,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>290</v>
       </c>
@@ -3012,7 +3015,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>291</v>
       </c>
@@ -3023,7 +3026,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>292</v>
       </c>
@@ -3034,7 +3037,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>293</v>
       </c>
@@ -3045,7 +3048,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>294</v>
       </c>
@@ -3056,7 +3059,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>295</v>
       </c>
@@ -3067,7 +3070,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -3078,7 +3081,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>297</v>
       </c>
@@ -3089,7 +3092,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>298</v>
       </c>
@@ -3100,7 +3103,7 @@
         <v>1055</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>299</v>
       </c>
@@ -3111,7 +3114,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>300</v>
       </c>
@@ -3122,7 +3125,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>301</v>
       </c>
@@ -3133,7 +3136,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>302</v>
       </c>
@@ -3144,7 +3147,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>303</v>
       </c>
@@ -3155,7 +3158,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>304</v>
       </c>
@@ -3166,7 +3169,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>305</v>
       </c>
@@ -3177,7 +3180,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>306</v>
       </c>
@@ -3188,7 +3191,7 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>307</v>
       </c>
@@ -3199,7 +3202,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>308</v>
       </c>
@@ -3210,7 +3213,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>309</v>
       </c>
@@ -3221,7 +3224,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>310</v>
       </c>
@@ -3232,7 +3235,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>311</v>
       </c>
@@ -3243,7 +3246,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>312</v>
       </c>
@@ -3254,7 +3257,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>313</v>
       </c>
@@ -3265,7 +3268,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>314</v>
       </c>
@@ -3276,7 +3279,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>315</v>
       </c>
@@ -3287,7 +3290,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>316</v>
       </c>
@@ -3298,7 +3301,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>317</v>
       </c>
@@ -3309,7 +3312,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>318</v>
       </c>
@@ -3320,7 +3323,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>319</v>
       </c>
@@ -3331,7 +3334,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>320</v>
       </c>
@@ -3342,7 +3345,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>321</v>
       </c>
@@ -3353,7 +3356,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>322</v>
       </c>
@@ -3364,7 +3367,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>323</v>
       </c>
@@ -3375,7 +3378,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>324</v>
       </c>
@@ -3386,7 +3389,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>325</v>
       </c>
@@ -3397,7 +3400,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>326</v>
       </c>
@@ -3408,7 +3411,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>327</v>
       </c>
@@ -3419,7 +3422,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>328</v>
       </c>
@@ -3430,7 +3433,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>329</v>
       </c>
@@ -3441,7 +3444,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>330</v>
       </c>
@@ -3452,7 +3455,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>331</v>
       </c>
@@ -3463,7 +3466,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>332</v>
       </c>
@@ -3474,7 +3477,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>333</v>
       </c>
@@ -3485,7 +3488,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>334</v>
       </c>
@@ -3496,7 +3499,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>335</v>
       </c>
@@ -3507,7 +3510,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>336</v>
       </c>
@@ -3529,9 +3532,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>286</v>
       </c>
@@ -3565,9 +3568,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:CZ2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:104" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3881,7 +3884,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="2" spans="1:104" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9844</v>
       </c>
@@ -4185,9 +4188,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>162</v>
       </c>
@@ -4240,7 +4243,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9844</v>
       </c>
@@ -4269,7 +4272,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9844</v>
       </c>
@@ -4304,7 +4307,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9844</v>
       </c>
@@ -4333,7 +4336,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9844</v>
       </c>
@@ -4383,7 +4386,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9844</v>
       </c>
@@ -4418,7 +4421,7 @@
         <v>135</v>
       </c>
       <c r="L6">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="M6" t="s">
         <v>5</v>
@@ -4433,7 +4436,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>9844</v>
       </c>
@@ -4468,7 +4471,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9844</v>
       </c>
@@ -4515,7 +4518,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9844</v>
       </c>
@@ -4544,7 +4547,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9844</v>
       </c>
@@ -4579,7 +4582,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9844</v>
       </c>
@@ -4614,7 +4617,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9844</v>
       </c>
@@ -4652,7 +4655,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:Q12" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:Q5 A9:Q12 A8:K8 M8:Q8 A7:Q7 A6:K6 M6:Q6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4660,9 +4663,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>162</v>
       </c>
@@ -4694,7 +4697,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9844</v>
       </c>
@@ -4717,7 +4720,7 @@
         <v>213</v>
       </c>
       <c r="H2">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="I2">
         <v>45372</v>
@@ -4726,7 +4729,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9844</v>
       </c>
@@ -4758,7 +4761,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9844</v>
       </c>
@@ -4781,7 +4784,7 @@
         <v>215</v>
       </c>
       <c r="H4">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="I4">
         <v>45373</v>
@@ -4793,7 +4796,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 A3:J3 A2:G2 I2:J2 A4:G4 I4:J4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4801,7 +4804,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4813,9 +4816,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>162</v>
       </c>
@@ -4847,7 +4850,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9844</v>
       </c>
@@ -4890,9 +4893,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>162</v>
       </c>
@@ -4909,7 +4912,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9844</v>
       </c>
@@ -4931,7 +4934,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4943,9 +4946,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:P37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>162</v>
       </c>
@@ -4995,7 +4998,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9844</v>
       </c>
@@ -5045,7 +5048,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9844</v>
       </c>
@@ -5095,7 +5098,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9844</v>
       </c>
@@ -5145,7 +5148,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9844</v>
       </c>
@@ -5195,7 +5198,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9844</v>
       </c>
@@ -5245,7 +5248,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>9844</v>
       </c>
@@ -5295,7 +5298,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9844</v>
       </c>
@@ -5345,7 +5348,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9844</v>
       </c>
@@ -5395,7 +5398,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9844</v>
       </c>
@@ -5445,7 +5448,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9844</v>
       </c>
@@ -5495,7 +5498,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9844</v>
       </c>
@@ -5545,7 +5548,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9844</v>
       </c>
@@ -5595,7 +5598,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>9844</v>
       </c>
@@ -5645,7 +5648,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9844</v>
       </c>
@@ -5695,7 +5698,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>9844</v>
       </c>
@@ -5745,7 +5748,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>9844</v>
       </c>
@@ -5795,7 +5798,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>9844</v>
       </c>
@@ -5845,7 +5848,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>9844</v>
       </c>
@@ -5895,7 +5898,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>9844</v>
       </c>
@@ -5945,7 +5948,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>9844</v>
       </c>
@@ -5995,7 +5998,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>9844</v>
       </c>
@@ -6045,7 +6048,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>9844</v>
       </c>
@@ -6095,7 +6098,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>9844</v>
       </c>
@@ -6145,7 +6148,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>9844</v>
       </c>
@@ -6195,7 +6198,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>9844</v>
       </c>
@@ -6245,7 +6248,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>9844</v>
       </c>
@@ -6295,7 +6298,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>9844</v>
       </c>
@@ -6345,7 +6348,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>9844</v>
       </c>
@@ -6395,7 +6398,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>9844</v>
       </c>
@@ -6445,7 +6448,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>9844</v>
       </c>
@@ -6495,7 +6498,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>9844</v>
       </c>
@@ -6545,7 +6548,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>9844</v>
       </c>
@@ -6595,7 +6598,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>9844</v>
       </c>
@@ -6645,7 +6648,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>9844</v>
       </c>
@@ -6695,7 +6698,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>9844</v>
       </c>
@@ -6745,7 +6748,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>9844</v>
       </c>

</xml_diff>